<commit_message>
Publish measured Studio evaluations and evidence-rich sample workbooks
</commit_message>
<xml_diff>
--- a/outputs/D_merged_wrapped.xlsx
+++ b/outputs/D_merged_wrapped.xlsx
@@ -12,13 +12,23 @@
     <sheet name="Page Audit" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Provenance" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Read me" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cell Evidence" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Verification" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Constraints" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Repair Proposals" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Correction History" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data 1'!$A$1:$D$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Validation Report'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Page Audit'!$A$1:$L$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Provenance'!$A$1:$E$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Read me'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Read me'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cell Evidence'!$A$1:$M$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Verification'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Constraints'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Repair Proposals'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Correction History'!$A$1:$I$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -537,6 +547,97 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D4"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C1" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId16"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Time UTC</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Excel row</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Before</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>After</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Previous hash</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Event hash</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -737,7 +838,7 @@
         <v>0.98</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.041</v>
+        <v>0.022</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -757,7 +858,7 @@
         <v>0</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>76.59999999999999</v>
+        <v>1076.6</v>
       </c>
       <c r="L2" s="2" t="inlineStr"/>
     </row>
@@ -885,10 +986,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="65" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -923,7 +1024,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.06</v>
+        <v>0.041</v>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
@@ -986,8 +1087,1316 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Cell evidence</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Ctrl+click a linked data cell for its source bounding box and original readings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Repair proposals</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Arithmetic-derived suggestions only. Source documents may contain errors. Never applied automatically.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Data sheet</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Excel row</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Source page</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>x0</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>y0</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>x1</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>y1</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>OCR score</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Initial reading</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="17" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>header</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="17" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>header</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>header</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>header</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>755</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>header</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>575</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>header</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>755</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>header</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>575</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>755</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>header</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Long product name</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>575</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>575</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>755</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>36.00</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Wrapped description</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>575</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>575</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>755</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>45.00</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>302</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>302</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>395</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>575</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>302</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>575</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>755</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>302</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>native-lines</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>30.00</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M21"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Source SHA-256</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>e8a441b23bca503cd5ea8a74044f47c89801ffbc4c93a9df136d9cf0ced3d042</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Extraction snapshot SHA-256</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>1be4598757131365cff6cf4f7b0dfbe590132779d30e12ca2347124e717f20f4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Review status</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Unreviewed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Review meaning</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>A human source-check attestation; not independent accuracy certification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Review note</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>cells with source boxes</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>equations</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>equation checks</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>failed equation checks</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>proposals with multiple equations</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Inferred relation</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Checked rows</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Matching rows</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Empirical agreement</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Violations</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Excel row</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Observed</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Supporting equations</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Caution</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Complete final extraction audit and release gates
</commit_message>
<xml_diff>
--- a/outputs/D_merged_wrapped.xlsx
+++ b/outputs/D_merged_wrapped.xlsx
@@ -22,15 +22,15 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data 1'!$A$1:$D$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Validation Report'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Page Audit'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Page Audit'!$A$1:$Q$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Join Receipt'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Provenance'!$A$1:$E$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Read me'!$A$1:$B$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cell Evidence'!$A$1:$O$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cell Evidence'!$A$1:$X$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Verification'!$A$1:$B$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Constraints'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Repair Proposals'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Correction History'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Correction History'!$A$1:$J$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -60,12 +60,17 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF0B3"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -85,18 +90,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -655,7 +663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,59 +673,65 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Evidence ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Time UTC</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Table</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Excel row</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Before</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>After</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Previous hash</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Event hash</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -736,9 +750,9 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="65" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="49" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -784,28 +798,32 @@
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>info</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>no_findings</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>No implemented rule raised a finding. This is not proof of accuracy.</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Compare with the source.</t>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="5" t="n"/>
+      <c r="E2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>layout_review</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Multi-level merged headers flattened into source-backed column paths.</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Verify the source page and reconstructed cells.</t>
         </is>
       </c>
     </row>
@@ -821,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -830,12 +848,17 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="65" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -871,79 +894,127 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Candidate ID</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Execution</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Selection reason</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Selected</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Tables</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Cells</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Findings</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Error</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="17" customHeight="1">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+    <row r="2" ht="51" customHeight="1">
+      <c r="A2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>digital</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="5" t="n">
         <v>0.98</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>0.018</v>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="E2" s="5" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>lines</t>
         </is>
       </c>
-      <c r="G2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" s="2" t="n">
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>p001-c01</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>native-primary</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>sequential</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Highest deterministic candidate key: trusted layout, credible content, structural quality, then validation-adjusted score; plan order breaks exact ties.</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="2" t="n">
+      <c r="O2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" s="5" t="n">
         <v>1076.6</v>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="Q2" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L2"/>
+  <autoFilter ref="A1:Q2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1010,32 +1081,32 @@
       </c>
     </row>
     <row r="2" ht="17" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="2" t="n">
+      <c r="F2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="5" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1089,63 +1160,63 @@
       </c>
     </row>
     <row r="2" ht="17" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="C2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
     </row>
     <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
     </row>
     <row r="4" ht="17" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="C4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
@@ -1183,142 +1254,142 @@
       </c>
     </row>
     <row r="2" ht="17" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>D_merged_wrapped.pdf</t>
         </is>
       </c>
     </row>
     <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Runtime seconds</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>0.047</v>
+      <c r="B3" s="5" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="4" ht="119" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Text encoding</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>All XLSX string fields use a reversible encoding: a literal backslash is doubled; XML-forbidden code points use a backslash followed by u and four hexadecimal digits. An underscore starting an OOXML escape-like sequence uses the same Unicode encoding. Decode left to right, treating each doubled backslash as one literal backslash. The full audit JSON and saved workspace retain the original strings.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="68" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Long text</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Values exceeding Excel's 32767-character cell limit show an explicit preview. The Long Text sheet preserves the complete encoded value in numbered chunks. Join its chunks in order before decoding the text encoding.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="68" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Small numbers</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Numbers below Excel's normal floating-point range remain exact text. Numbers needing more than 12 decimal places use General formatting; percentages needing more than 12 display decimals remain text, avoiding a false zero.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Yellow cells</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Review required. See Validation Report for the reason and source row.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Source row</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Data row within the extracted source table, excluding detected headers.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Extraction heuristic / OCR score, not a calibrated probability of correctness.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Dates</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>ISO and unambiguous day-first dates are typed. Ambiguous dates stay text.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Source strings are stored as text. No source formulas are executed.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Cell evidence</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Ctrl+click a linked data cell for its source bounding box and original readings.</t>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Ctrl+click a linked data cell for its source box, confidence meaning, original readings, alternatives and correction count.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Repair proposals</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Arithmetic-derived suggestions only. Source documents may contain errors. Never applied automatically.</t>
         </is>
@@ -1336,1205 +1407,2039 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
     <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="65" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="58" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="65" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Evidence ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Data sheet</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Excel row</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Working value</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Original extracted value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Original source reading</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Source page</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>x0</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>y0</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>x1</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>y1</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Engine</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>OCR score</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence type</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Recognition score</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence meaning</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Reading</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Initial reading</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence state</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Location status</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Location reason</t>
         </is>
       </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Corrections</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Alternative readings</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="17" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>T1:H:C1</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="n">
+      <c r="C2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Product | Code</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Product | Code</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Product | Code</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="J2" s="5" t="n">
         <v>92</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="K2" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="L2" s="5" t="n">
         <v>134</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="n"/>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>header</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="R2" s="5" t="inlineStr"/>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>merged_header_path</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="V2" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="5" t="inlineStr"/>
     </row>
     <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>T1:H:C1</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="2" t="n">
+      <c r="C3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Product | Code</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Product | Code</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Product | Code</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="J3" s="5" t="n">
         <v>134</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="K3" s="5" t="n">
         <v>215</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="L3" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="n"/>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>header</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="R3" s="5" t="inlineStr"/>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>merged_header_path</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="V3" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="5" t="inlineStr"/>
     </row>
     <row r="4" ht="17" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>T1:H:C2</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Product | Description</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Product | Description</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Product | Description</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="J4" s="5" t="n">
         <v>92</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="K4" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="L4" s="5" t="n">
         <v>134</v>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="n"/>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>header</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="R4" s="5" t="inlineStr"/>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>merged_header_path</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="V4" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="5" t="inlineStr"/>
     </row>
     <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>T1:H:C2</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Product | Description</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Product | Description</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Product | Description</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="5" t="n">
         <v>215</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="J5" s="5" t="n">
         <v>134</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="K5" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="L5" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n"/>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="n"/>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>header</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="R5" s="5" t="inlineStr"/>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>merged_header_path</t>
+        </is>
+      </c>
+      <c r="T5" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U5" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="V5" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>T1:H:C3</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Units</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Units</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Units</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="J6" s="5" t="n">
         <v>92</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="K6" s="5" t="n">
         <v>755</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="L6" s="5" t="n">
         <v>134</v>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="n"/>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr">
         <is>
           <t>Movement</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>header</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="R6" s="5" t="inlineStr"/>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>merged_header_path</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="V6" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>T1:H:C3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Units</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Units</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Units</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="J7" s="5" t="n">
         <v>134</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="K7" s="5" t="n">
         <v>575</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="L7" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="M7" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="n"/>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>header</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="R7" s="5" t="inlineStr"/>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>merged_header_path</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="V7" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>T1:H:C4</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Value</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Value</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Value</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="J8" s="5" t="n">
         <v>92</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="K8" s="5" t="n">
         <v>755</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="L8" s="5" t="n">
         <v>134</v>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="n"/>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
         <is>
           <t>Movement</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>header</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="R8" s="5" t="inlineStr"/>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>merged_header_path</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="V8" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>T1:H:C4</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Value</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Value</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Movement | Value</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="5" t="n">
         <v>575</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="J9" s="5" t="n">
         <v>134</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="K9" s="5" t="n">
         <v>755</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="L9" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="n"/>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>header</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="R9" s="5" t="inlineStr"/>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>merged_header_path</t>
+        </is>
+      </c>
+      <c r="T9" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U9" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="V9" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>T1:R1:C1</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="C10" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="2" t="n">
+      <c r="D10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="J10" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="K10" s="5" t="n">
         <v>215</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="L10" s="5" t="n">
         <v>218</v>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="n"/>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
         <is>
           <t>A01</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="R10" s="5" t="inlineStr"/>
+      <c r="S10" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U10" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="V10" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>T1:R1:C2</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="C11" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="D11" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Long product name</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Long product name</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Long product name</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="5" t="n">
         <v>215</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="J11" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="K11" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="L11" s="5" t="n">
         <v>218</v>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="M11" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="n"/>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
         <is>
           <t>Long product name</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="R11" s="5" t="inlineStr"/>
+      <c r="S11" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="V11" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>T1:R1:C3</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="C12" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="D12" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="J12" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="K12" s="5" t="n">
         <v>575</v>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="L12" s="5" t="n">
         <v>218</v>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="M12" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n"/>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="n"/>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="R12" s="5" t="inlineStr"/>
+      <c r="S12" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="V12" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>T1:R1:C4</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="C13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="D13" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>36.00</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>36.00</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>36.00</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="5" t="n">
         <v>575</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="J13" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="K13" s="5" t="n">
         <v>755</v>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="L13" s="5" t="n">
         <v>218</v>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="M13" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="n"/>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
         <is>
           <t>36.00</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="R13" s="5" t="inlineStr"/>
+      <c r="S13" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="V13" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="5" t="inlineStr"/>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>T1:R2:C1</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="C14" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="2" t="n">
+      <c r="D14" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="J14" s="5" t="n">
         <v>218</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="K14" s="5" t="n">
         <v>215</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="L14" s="5" t="n">
         <v>260</v>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="M14" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n"/>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="n"/>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
         <is>
           <t>A02</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="R14" s="5" t="inlineStr"/>
+      <c r="S14" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="T14" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U14" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="V14" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="5" t="inlineStr"/>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>T1:R2:C2</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="C15" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="D15" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Wrapped description</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Wrapped description</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Wrapped description</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="5" t="n">
         <v>215</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="J15" s="5" t="n">
         <v>218</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="K15" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="L15" s="5" t="n">
         <v>260</v>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="M15" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n"/>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="n"/>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
         <is>
           <t>Wrapped description</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="R15" s="5" t="inlineStr"/>
+      <c r="S15" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="T15" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U15" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr">
+      <c r="V15" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>T1:R2:C3</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="C16" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="D16" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="J16" s="5" t="n">
         <v>218</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="K16" s="5" t="n">
         <v>575</v>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="L16" s="5" t="n">
         <v>260</v>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="M16" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J16" s="2" t="n"/>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="n"/>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="R16" s="5" t="inlineStr"/>
+      <c r="S16" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U16" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="V16" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="5" t="inlineStr"/>
     </row>
     <row r="17" ht="17" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>T1:R2:C4</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="C17" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C17" s="2" t="n">
+      <c r="D17" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>45.00</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>45.00</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>45.00</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="5" t="n">
         <v>575</v>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="J17" s="5" t="n">
         <v>218</v>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="K17" s="5" t="n">
         <v>755</v>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="L17" s="5" t="n">
         <v>260</v>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="M17" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J17" s="2" t="n"/>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="n"/>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
         <is>
           <t>45.00</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="R17" s="5" t="inlineStr"/>
+      <c r="S17" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="T17" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U17" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="V17" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" s="5" t="inlineStr"/>
     </row>
     <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>T1:R3:C1</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="C18" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="C18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="2" t="n">
+      <c r="D18" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="J18" s="5" t="n">
         <v>260</v>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="K18" s="5" t="n">
         <v>215</v>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="L18" s="5" t="n">
         <v>302</v>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="M18" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J18" s="2" t="n"/>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="n"/>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
         <is>
           <t>A03</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="R18" s="5" t="inlineStr"/>
+      <c r="S18" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U18" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="V18" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" s="5" t="inlineStr"/>
     </row>
     <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>T1:R3:C2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="C19" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="D19" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="5" t="n">
         <v>215</v>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="J19" s="5" t="n">
         <v>260</v>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="K19" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="H19" s="2" t="n">
+      <c r="L19" s="5" t="n">
         <v>302</v>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="M19" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J19" s="2" t="n"/>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="n"/>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="R19" s="5" t="inlineStr"/>
+      <c r="S19" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U19" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="V19" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" s="5" t="inlineStr"/>
     </row>
     <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>T1:R3:C3</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="C20" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="D20" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="5" t="n">
         <v>395</v>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="J20" s="5" t="n">
         <v>260</v>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="K20" s="5" t="n">
         <v>575</v>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="L20" s="5" t="n">
         <v>302</v>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="M20" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="n"/>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="R20" s="5" t="inlineStr"/>
+      <c r="S20" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="T20" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U20" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr">
+      <c r="V20" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" s="5" t="inlineStr"/>
     </row>
     <row r="21" ht="17" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>T1:R3:C4</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Data 1</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="C21" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="C21" s="2" t="n">
+      <c r="D21" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="2" t="n">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>30.00</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>30.00</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>30.00</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="5" t="n">
         <v>575</v>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="J21" s="5" t="n">
         <v>260</v>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="K21" s="5" t="n">
         <v>755</v>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="L21" s="5" t="n">
         <v>302</v>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="M21" s="5" t="inlineStr">
         <is>
           <t>native-lines</t>
         </is>
       </c>
-      <c r="J21" s="2" t="n"/>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>native_text</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="n"/>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>Text and geometry came directly from the PDF text layer.</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
         <is>
           <t>30.00</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="R21" s="5" t="inlineStr"/>
+      <c r="S21" s="5" t="inlineStr">
         <is>
           <t>extracted</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="T21" s="5" t="inlineStr">
+        <is>
+          <t>exact_source_box</t>
+        </is>
+      </c>
+      <c r="U21" s="5" t="inlineStr">
         <is>
           <t>located</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="V21" s="5" t="inlineStr">
         <is>
           <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
+      <c r="W21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X21" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O21"/>
+  <autoFilter ref="A1:X21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2565,170 +3470,170 @@
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Source SHA-256</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>e8a441b23bca503cd5ea8a74044f47c89801ffbc4c93a9df136d9cf0ced3d042</t>
         </is>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Extraction snapshot SHA-256</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>c3e6977187cbb687afb0789c7f4dc5b39685feed409fd7304162c662f16cd737</t>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>e9d79857e0c2336a685d6eea44bd3dcd8d2d923e1c7b40e2eb6c82ba304f490c</t>
         </is>
       </c>
     </row>
     <row r="4" ht="17" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Review status</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Unreviewed</t>
         </is>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Review meaning</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>A human source-check attestation; not independent accuracy certification.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Review note</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Export type</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Draft Excel</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Non-empty exported cells</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="5" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Cells with source boxes</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="5" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Cells requiring full-page evidence review</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Cell source-box coverage</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>cells</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="5" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>cells with source boxes</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="5" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>equations</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>equation checks</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>failed equation checks</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B16" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>proposals with multiple equations</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" s="5" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>